<commit_message>
Rebuild CFI templates from originals with authentic FICO inputs
Restore pristine CFI 3-statement and DCF workbooks, fill the real
input cells with SEC FICO numbers, and regenerate the linked MEGA file.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/DCF resources/CFI_3-Statement-Model-Complete.xlsx
+++ b/DCF resources/CFI_3-Statement-Model-Complete.xlsx
@@ -609,7 +609,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -837,7 +837,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -885,7 +885,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -923,7 +923,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1003,7 +1003,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1208,7 +1208,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1256,7 +1256,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1294,7 +1294,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -1315,6 +1315,54 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>714374</colOff>
+      <row>3</row>
+      <rowOff>19050</rowOff>
+    </from>
+    <to>
+      <col>4</col>
+      <colOff>661827</colOff>
+      <row>9</row>
+      <rowOff>114300</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Picture 1">
+          <a:hlinkClick r:id="rId1"/>
+        </cNvPr>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="1447799" y="762000"/>
+          <a:ext cx="3359943" cy="1581150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
@@ -1368,6 +1416,49 @@
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>1</col>
+      <colOff>38101</colOff>
+      <row>131</row>
+      <rowOff>129314</rowOff>
+    </from>
+    <to>
+      <col>1</col>
+      <colOff>783591</colOff>
+      <row>135</row>
+      <rowOff>144144</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Picture 3">
+          <a:hlinkClick r:id="rId1"/>
+        </cNvPr>
+        <cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm>
+          <a:off x="647701" y="5158514"/>
+          <a:ext cx="742950" cy="813659"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
     <clientData/>
   </twoCellAnchor>
 </wsDr>
@@ -1801,7 +1892,7 @@
       <c r="B12" s="74" t="n"/>
       <c r="C12" s="75" t="inlineStr">
         <is>
-          <t>FICO — 3 Statement Model (CFI template, populated)</t>
+          <t>FICO — 3 Statement Model</t>
         </is>
       </c>
       <c r="D12" s="74" t="n"/>
@@ -1949,7 +2040,7 @@
       <c r="B20" s="85" t="n"/>
       <c r="C20" s="86" t="inlineStr">
         <is>
-          <t>Simplified FICO mapping into CFI 3-statement structure (no goodwill/other assets). Educational use only.</t>
+          <t>Populated with Fair Isaac Corp (FICO) SEC 10-K numbers. Units: $ thousands. Educational only.</t>
         </is>
       </c>
       <c r="D20" s="86" t="n"/>
@@ -1969,7 +2060,7 @@
       <c r="B21" s="85" t="n"/>
       <c r="C21" s="85" t="inlineStr">
         <is>
-          <t>Historical FY2021-FY2025 from SEC 10-K/XBRL; forecast FY2026-FY2030 base case. Units: $ thousands.</t>
+          <t>Yellow/blue cells = inputs. History FY2021–FY2025; forecast FY2026–FY2030.</t>
         </is>
       </c>
       <c r="D21" s="85" t="n"/>
@@ -2157,6 +2248,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" scale="64"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2166,7 +2258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N138"/>
+  <dimension ref="A1:U138"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="15.6" outlineLevelRow="1"/>
   <cols>
     <col width="1.88671875" customWidth="1" style="19" min="1" max="1"/>
@@ -2301,6 +2393,7 @@
         <v/>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="65" t="inlineStr">
         <is>
@@ -2416,7 +2509,7 @@
     <row r="9" hidden="1" outlineLevel="1">
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>SG&amp;A + R&amp;D + other opex, ex-D&amp;A ($000's)</t>
+          <t>SG&amp;A ($000's)</t>
         </is>
       </c>
       <c r="C9" s="19" t="n"/>
@@ -2442,25 +2535,25 @@
         <v/>
       </c>
       <c r="J9" s="93" t="n">
-        <v>794973.3</v>
+        <v>584851.9</v>
       </c>
       <c r="K9" s="93" t="n">
-        <v>781026.4</v>
+        <v>574591.4</v>
       </c>
       <c r="L9" s="93" t="n">
-        <v>767079.5</v>
+        <v>564330.8</v>
       </c>
       <c r="M9" s="93" t="n">
-        <v>760106.1</v>
+        <v>559200.5</v>
       </c>
       <c r="N9" s="93" t="n">
-        <v>753132.6</v>
+        <v>554070.2</v>
       </c>
     </row>
     <row r="10" hidden="1" outlineLevel="1">
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Other income (as negative overhead) ($000's)</t>
+          <t>R&amp;D + other opex residual ($000's)</t>
         </is>
       </c>
       <c r="C10" s="19" t="n"/>
@@ -2486,19 +2579,19 @@
         <v/>
       </c>
       <c r="J10" s="93" t="n">
-        <v>0</v>
+        <v>210121.4</v>
       </c>
       <c r="K10" s="93" t="n">
-        <v>0</v>
+        <v>206435</v>
       </c>
       <c r="L10" s="93" t="n">
-        <v>0</v>
+        <v>202748.7</v>
       </c>
       <c r="M10" s="93" t="n">
-        <v>0</v>
+        <v>200905.5</v>
       </c>
       <c r="N10" s="93" t="n">
-        <v>0</v>
+        <v>199062.4</v>
       </c>
     </row>
     <row r="11" hidden="1" outlineLevel="1">
@@ -2530,19 +2623,19 @@
         <v/>
       </c>
       <c r="J11" s="92" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="K11" s="92" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="L11" s="92" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="M11" s="92" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="N11" s="92" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" hidden="1" outlineLevel="1">
@@ -2953,7 +3046,7 @@
     <row r="24" hidden="1" outlineLevel="1">
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Reveneue</t>
         </is>
       </c>
       <c r="C24" s="18" t="n"/>
@@ -3109,23 +3202,23 @@
     <row r="28" hidden="1" outlineLevel="1">
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>SG&amp;A + R&amp;D + other opex (ex-D&amp;A)</t>
+          <t>SG&amp;A</t>
         </is>
       </c>
       <c r="E28" s="93" t="n">
-        <v>452993</v>
+        <v>396281</v>
       </c>
       <c r="F28" s="93" t="n">
-        <v>512217</v>
+        <v>383863</v>
       </c>
       <c r="G28" s="93" t="n">
-        <v>545036</v>
+        <v>400565</v>
       </c>
       <c r="H28" s="93" t="n">
-        <v>621864</v>
+        <v>462834</v>
       </c>
       <c r="I28" s="93" t="n">
-        <v>697345</v>
+        <v>513028</v>
       </c>
       <c r="J28" s="19">
         <f>J9</f>
@@ -3151,23 +3244,23 @@
     <row r="29" hidden="1" outlineLevel="1">
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Other income, net (negative = income)</t>
+          <t>R&amp;D + other opex residual</t>
         </is>
       </c>
       <c r="E29" s="93" t="n">
-        <v>0</v>
+        <v>56712</v>
       </c>
       <c r="F29" s="93" t="n">
-        <v>0</v>
+        <v>128354</v>
       </c>
       <c r="G29" s="93" t="n">
-        <v>-6340</v>
+        <v>144471</v>
       </c>
       <c r="H29" s="93" t="n">
-        <v>-14034</v>
+        <v>159030</v>
       </c>
       <c r="I29" s="93" t="n">
-        <v>-11392</v>
+        <v>184317</v>
       </c>
       <c r="J29" s="19">
         <f>J10</f>
@@ -4606,19 +4699,19 @@
         </is>
       </c>
       <c r="E73" s="93" t="n">
-        <v>0</v>
+        <v>-661519</v>
       </c>
       <c r="F73" s="93" t="n">
-        <v>0</v>
+        <v>-1251001</v>
       </c>
       <c r="G73" s="93" t="n">
-        <v>0</v>
+        <v>-360388</v>
       </c>
       <c r="H73" s="93" t="n">
-        <v>0</v>
+        <v>-849330</v>
       </c>
       <c r="I73" s="93" t="n">
-        <v>0</v>
+        <v>-1398028</v>
       </c>
       <c r="J73" s="19">
         <f>J20</f>
@@ -5794,14 +5887,14 @@
     <row r="131">
       <c r="B131" s="95" t="inlineStr">
         <is>
-          <t>FICO simplified 3-statement mapping — educational only. Goodwill, deferred revenue, leases, SBC and buybacks not fully modeled.</t>
+          <t>FICO mapping: Revenue/COGS/Interest/Tax from 10-K; SG&amp;A→Salaries; R&amp;D residual→Rent so OpInc identity holds.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="B132" s="95" t="inlineStr">
         <is>
-          <t>Yellow/blue cells = FICO inputs. Forecast J-N: growth 14%→8%, EBIT-like opex via SG&amp;A+R&amp;D, tax 18.8%, kd 5.5%, AR days ~97.</t>
+          <t>Template BS is simplified (Cash/AR/Inv/PPE vs AP/Debt). Equity is a plug. Yellow/blue = inputs.</t>
         </is>
       </c>
       <c r="C132" s="69" t="n"/>
@@ -5810,7 +5903,7 @@
     <row r="133">
       <c r="B133" s="95" t="inlineStr">
         <is>
-          <t>Sources: SEC EDGAR FY2025 10-K / companyfacts; market bridge uses 10-Q 2026-06-30 in the DCF file.</t>
+          <t>Sources: SEC EDGAR FY2025 10-K / companyfacts; forecast drivers are base-case assumptions.</t>
         </is>
       </c>
       <c r="C133" s="69" t="n"/>

</xml_diff>

<commit_message>
Add SEC-driven FICO_DCF_Financial_Model from CFI blueprints
Add build_fico_model.py that pulls FICO 10-K companyfacts from EDGAR,
injects historicals into pristine CFI 3-statement/DCF input cells only,
preserves native formulas, and writes FICO_DCF_Financial_Model.xlsx.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/DCF resources/CFI_3-Statement-Model-Complete.xlsx
+++ b/DCF resources/CFI_3-Statement-Model-Complete.xlsx
@@ -364,7 +364,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
@@ -511,9 +511,13 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
     <xf numFmtId="0" fontId="25" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="7"/>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="166" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="164" fontId="26" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="26" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="26" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="9">
@@ -1892,7 +1896,7 @@
       <c r="B12" s="74" t="n"/>
       <c r="C12" s="75" t="inlineStr">
         <is>
-          <t>FICO — 3 Statement Model</t>
+          <t>FICO — 3 Statement Model (CFI template)</t>
         </is>
       </c>
       <c r="D12" s="74" t="n"/>
@@ -2040,7 +2044,7 @@
       <c r="B20" s="85" t="n"/>
       <c r="C20" s="86" t="inlineStr">
         <is>
-          <t>Populated with Fair Isaac Corp (FICO) SEC 10-K numbers. Units: $ thousands. Educational only.</t>
+          <t>Historical inputs from SEC EDGAR 10-K. Forecast formulas preserved.</t>
         </is>
       </c>
       <c r="D20" s="86" t="n"/>
@@ -2060,7 +2064,7 @@
       <c r="B21" s="85" t="n"/>
       <c r="C21" s="85" t="inlineStr">
         <is>
-          <t>Yellow/blue cells = inputs. History FY2021–FY2025; forecast FY2026–FY2030.</t>
+          <t>All content is Copyright material of CFI Education Inc.</t>
         </is>
       </c>
       <c r="D21" s="85" t="n"/>
@@ -2306,7 +2310,7 @@
       </c>
       <c r="C2" s="62" t="n"/>
       <c r="D2" s="63" t="n"/>
-      <c r="E2" s="83" t="n">
+      <c r="E2" s="92" t="n">
         <v>2021</v>
       </c>
       <c r="F2" s="83">
@@ -2446,19 +2450,19 @@
         <f>I24/H24-1</f>
         <v/>
       </c>
-      <c r="J7" s="92" t="n">
+      <c r="J7" s="93" t="n">
         <v>0.14</v>
       </c>
-      <c r="K7" s="92" t="n">
+      <c r="K7" s="93" t="n">
         <v>0.12</v>
       </c>
-      <c r="L7" s="92" t="n">
+      <c r="L7" s="93" t="n">
         <v>0.1</v>
       </c>
-      <c r="M7" s="92" t="n">
+      <c r="M7" s="93" t="n">
         <v>0.09</v>
       </c>
-      <c r="N7" s="92" t="n">
+      <c r="N7" s="93" t="n">
         <v>0.08</v>
       </c>
     </row>
@@ -2490,20 +2494,20 @@
         <f>I25/I24</f>
         <v/>
       </c>
-      <c r="J8" s="92" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="K8" s="92" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="L8" s="92" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="M8" s="92" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="N8" s="92" t="n">
-        <v>0.17</v>
+      <c r="J8" s="93" t="n">
+        <v>0.1777</v>
+      </c>
+      <c r="K8" s="93" t="n">
+        <v>0.1777</v>
+      </c>
+      <c r="L8" s="93" t="n">
+        <v>0.1777</v>
+      </c>
+      <c r="M8" s="93" t="n">
+        <v>0.1777</v>
+      </c>
+      <c r="N8" s="93" t="n">
+        <v>0.1777</v>
       </c>
     </row>
     <row r="9" hidden="1" outlineLevel="1">
@@ -2534,26 +2538,26 @@
         <f>I28</f>
         <v/>
       </c>
-      <c r="J9" s="93" t="n">
+      <c r="J9" s="94" t="n">
         <v>584851.9</v>
       </c>
-      <c r="K9" s="93" t="n">
+      <c r="K9" s="94" t="n">
         <v>574591.4</v>
       </c>
-      <c r="L9" s="93" t="n">
+      <c r="L9" s="94" t="n">
         <v>564330.8</v>
       </c>
-      <c r="M9" s="93" t="n">
+      <c r="M9" s="94" t="n">
         <v>559200.5</v>
       </c>
-      <c r="N9" s="93" t="n">
+      <c r="N9" s="94" t="n">
         <v>554070.2</v>
       </c>
     </row>
     <row r="10" hidden="1" outlineLevel="1">
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>R&amp;D + other opex residual ($000's)</t>
+          <t>R&amp;D ($000's)</t>
         </is>
       </c>
       <c r="C10" s="19" t="n"/>
@@ -2578,20 +2582,20 @@
         <f>I29</f>
         <v/>
       </c>
-      <c r="J10" s="93" t="n">
-        <v>210121.4</v>
-      </c>
-      <c r="K10" s="93" t="n">
-        <v>206435</v>
-      </c>
-      <c r="L10" s="93" t="n">
-        <v>202748.7</v>
-      </c>
-      <c r="M10" s="93" t="n">
-        <v>200905.5</v>
-      </c>
-      <c r="N10" s="93" t="n">
-        <v>199062.4</v>
+      <c r="J10" s="94" t="n">
+        <v>214715.6</v>
+      </c>
+      <c r="K10" s="94" t="n">
+        <v>210948.6</v>
+      </c>
+      <c r="L10" s="94" t="n">
+        <v>207181.7</v>
+      </c>
+      <c r="M10" s="94" t="n">
+        <v>205298.2</v>
+      </c>
+      <c r="N10" s="94" t="n">
+        <v>203414.8</v>
       </c>
     </row>
     <row r="11" hidden="1" outlineLevel="1">
@@ -2622,20 +2626,20 @@
         <f>I30/I92</f>
         <v/>
       </c>
-      <c r="J11" s="92" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="K11" s="92" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="L11" s="92" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M11" s="92" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N11" s="92" t="n">
-        <v>0.25</v>
+      <c r="J11" s="93" t="n">
+        <v>0.3887</v>
+      </c>
+      <c r="K11" s="93" t="n">
+        <v>0.3887</v>
+      </c>
+      <c r="L11" s="93" t="n">
+        <v>0.3887</v>
+      </c>
+      <c r="M11" s="93" t="n">
+        <v>0.3887</v>
+      </c>
+      <c r="N11" s="93" t="n">
+        <v>0.3887</v>
       </c>
     </row>
     <row r="12" hidden="1" outlineLevel="1">
@@ -2666,20 +2670,20 @@
         <f>I101/I98</f>
         <v/>
       </c>
-      <c r="J12" s="92" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="K12" s="92" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="L12" s="92" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="M12" s="92" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="N12" s="92" t="n">
-        <v>0.055</v>
+      <c r="J12" s="93" t="n">
+        <v>0.0437</v>
+      </c>
+      <c r="K12" s="93" t="n">
+        <v>0.0437</v>
+      </c>
+      <c r="L12" s="93" t="n">
+        <v>0.0437</v>
+      </c>
+      <c r="M12" s="93" t="n">
+        <v>0.0437</v>
+      </c>
+      <c r="N12" s="93" t="n">
+        <v>0.0437</v>
       </c>
     </row>
     <row r="13" hidden="1" outlineLevel="1">
@@ -2710,20 +2714,20 @@
         <f>I35/I33</f>
         <v/>
       </c>
-      <c r="J13" s="92" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="K13" s="92" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="L13" s="92" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="M13" s="92" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="N13" s="92" t="n">
-        <v>0.188</v>
+      <c r="J13" s="93" t="n">
+        <v>0.1877</v>
+      </c>
+      <c r="K13" s="93" t="n">
+        <v>0.1877</v>
+      </c>
+      <c r="L13" s="93" t="n">
+        <v>0.1877</v>
+      </c>
+      <c r="M13" s="93" t="n">
+        <v>0.1877</v>
+      </c>
+      <c r="N13" s="93" t="n">
+        <v>0.1877</v>
       </c>
     </row>
     <row r="14" hidden="1" outlineLevel="1">
@@ -2772,19 +2776,19 @@
         <f>I42/I24*365</f>
         <v/>
       </c>
-      <c r="J15" s="93" t="n">
+      <c r="J15" s="94" t="n">
         <v>97</v>
       </c>
-      <c r="K15" s="93" t="n">
+      <c r="K15" s="94" t="n">
         <v>97</v>
       </c>
-      <c r="L15" s="93" t="n">
+      <c r="L15" s="94" t="n">
         <v>97</v>
       </c>
-      <c r="M15" s="93" t="n">
+      <c r="M15" s="94" t="n">
         <v>97</v>
       </c>
-      <c r="N15" s="93" t="n">
+      <c r="N15" s="94" t="n">
         <v>97</v>
       </c>
     </row>
@@ -2815,19 +2819,19 @@
         <f>I43/I25*365</f>
         <v/>
       </c>
-      <c r="J16" s="93" t="n">
+      <c r="J16" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="93" t="n">
+      <c r="K16" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="93" t="n">
+      <c r="L16" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="93" t="n">
+      <c r="M16" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="93" t="n">
+      <c r="N16" s="94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2858,20 +2862,20 @@
         <f>I48/I25*365</f>
         <v/>
       </c>
-      <c r="J17" s="93" t="n">
-        <v>33</v>
-      </c>
-      <c r="K17" s="93" t="n">
-        <v>33</v>
-      </c>
-      <c r="L17" s="93" t="n">
-        <v>33</v>
-      </c>
-      <c r="M17" s="93" t="n">
-        <v>33</v>
-      </c>
-      <c r="N17" s="93" t="n">
-        <v>33</v>
+      <c r="J17" s="94" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="K17" s="94" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="L17" s="94" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="M17" s="94" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="N17" s="94" t="n">
+        <v>33.3</v>
       </c>
     </row>
     <row r="18" hidden="1" outlineLevel="1">
@@ -2900,19 +2904,19 @@
         <f>I68</f>
         <v/>
       </c>
-      <c r="J18" s="93" t="n">
+      <c r="J18" s="94" t="n">
         <v>45391.8</v>
       </c>
-      <c r="K18" s="93" t="n">
+      <c r="K18" s="94" t="n">
         <v>50838.8</v>
       </c>
-      <c r="L18" s="93" t="n">
+      <c r="L18" s="94" t="n">
         <v>55922.7</v>
       </c>
-      <c r="M18" s="93" t="n">
+      <c r="M18" s="94" t="n">
         <v>60955.8</v>
       </c>
-      <c r="N18" s="93" t="n">
+      <c r="N18" s="94" t="n">
         <v>65832.2</v>
       </c>
     </row>
@@ -2942,19 +2946,19 @@
         <f>I99</f>
         <v/>
       </c>
-      <c r="J19" s="93" t="n">
+      <c r="J19" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="93" t="n">
+      <c r="K19" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="L19" s="93" t="n">
+      <c r="L19" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="M19" s="93" t="n">
+      <c r="M19" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="93" t="n">
+      <c r="N19" s="94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2984,19 +2988,19 @@
         <f>I73</f>
         <v/>
       </c>
-      <c r="J20" s="93" t="n">
+      <c r="J20" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="93" t="n">
+      <c r="K20" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="L20" s="93" t="n">
+      <c r="L20" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="M20" s="93" t="n">
+      <c r="M20" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="93" t="n">
+      <c r="N20" s="94" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3051,19 +3055,19 @@
       </c>
       <c r="C24" s="18" t="n"/>
       <c r="D24" s="46" t="n"/>
-      <c r="E24" s="93" t="n">
+      <c r="E24" s="94" t="n">
         <v>1316536</v>
       </c>
-      <c r="F24" s="93" t="n">
+      <c r="F24" s="94" t="n">
         <v>1377270</v>
       </c>
-      <c r="G24" s="93" t="n">
+      <c r="G24" s="94" t="n">
         <v>1513557</v>
       </c>
-      <c r="H24" s="93" t="n">
+      <c r="H24" s="94" t="n">
         <v>1717526</v>
       </c>
-      <c r="I24" s="93" t="n">
+      <c r="I24" s="94" t="n">
         <v>1990869</v>
       </c>
       <c r="J24" s="18">
@@ -3095,19 +3099,19 @@
       </c>
       <c r="C25" s="19" t="n"/>
       <c r="D25" s="47" t="n"/>
-      <c r="E25" s="93" t="n">
+      <c r="E25" s="94" t="n">
         <v>332462</v>
       </c>
-      <c r="F25" s="93" t="n">
+      <c r="F25" s="94" t="n">
         <v>302174</v>
       </c>
-      <c r="G25" s="93" t="n">
+      <c r="G25" s="94" t="n">
         <v>311053</v>
       </c>
-      <c r="H25" s="93" t="n">
+      <c r="H25" s="94" t="n">
         <v>348206</v>
       </c>
-      <c r="I25" s="93" t="n">
+      <c r="I25" s="94" t="n">
         <v>353722</v>
       </c>
       <c r="J25" s="55">
@@ -3205,19 +3209,19 @@
           <t>SG&amp;A</t>
         </is>
       </c>
-      <c r="E28" s="93" t="n">
+      <c r="E28" s="94" t="n">
         <v>396281</v>
       </c>
-      <c r="F28" s="93" t="n">
+      <c r="F28" s="94" t="n">
         <v>383863</v>
       </c>
-      <c r="G28" s="93" t="n">
+      <c r="G28" s="94" t="n">
         <v>400565</v>
       </c>
-      <c r="H28" s="93" t="n">
+      <c r="H28" s="94" t="n">
         <v>462834</v>
       </c>
-      <c r="I28" s="93" t="n">
+      <c r="I28" s="94" t="n">
         <v>513028</v>
       </c>
       <c r="J28" s="19">
@@ -3244,23 +3248,23 @@
     <row r="29" hidden="1" outlineLevel="1">
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>R&amp;D + other opex residual</t>
-        </is>
-      </c>
-      <c r="E29" s="93" t="n">
-        <v>56712</v>
-      </c>
-      <c r="F29" s="93" t="n">
-        <v>128354</v>
-      </c>
-      <c r="G29" s="93" t="n">
-        <v>144471</v>
-      </c>
-      <c r="H29" s="93" t="n">
-        <v>159030</v>
-      </c>
-      <c r="I29" s="93" t="n">
-        <v>184317</v>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="E29" s="94" t="n">
+        <v>171231</v>
+      </c>
+      <c r="F29" s="94" t="n">
+        <v>146758</v>
+      </c>
+      <c r="G29" s="94" t="n">
+        <v>159950</v>
+      </c>
+      <c r="H29" s="94" t="n">
+        <v>171940</v>
+      </c>
+      <c r="I29" s="94" t="n">
+        <v>188347</v>
       </c>
       <c r="J29" s="19">
         <f>J10</f>
@@ -3289,19 +3293,19 @@
           <t>Depreciation &amp; Amortization</t>
         </is>
       </c>
-      <c r="E30" s="93" t="n">
+      <c r="E30" s="94" t="n">
         <v>25592</v>
       </c>
-      <c r="F30" s="93" t="n">
+      <c r="F30" s="94" t="n">
         <v>20465</v>
       </c>
-      <c r="G30" s="93" t="n">
+      <c r="G30" s="94" t="n">
         <v>14638</v>
       </c>
-      <c r="H30" s="93" t="n">
+      <c r="H30" s="94" t="n">
         <v>13827</v>
       </c>
-      <c r="I30" s="93" t="n">
+      <c r="I30" s="94" t="n">
         <v>14952</v>
       </c>
       <c r="J30" s="19">
@@ -3333,19 +3337,19 @@
       </c>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="24" t="n"/>
-      <c r="E31" s="94" t="n">
+      <c r="E31" s="95" t="n">
         <v>40092</v>
       </c>
-      <c r="F31" s="94" t="n">
+      <c r="F31" s="95" t="n">
         <v>68967</v>
       </c>
-      <c r="G31" s="94" t="n">
+      <c r="G31" s="95" t="n">
         <v>95546</v>
       </c>
-      <c r="H31" s="94" t="n">
+      <c r="H31" s="95" t="n">
         <v>105638</v>
       </c>
-      <c r="I31" s="94" t="n">
+      <c r="I31" s="95" t="n">
         <v>133647</v>
       </c>
       <c r="J31" s="16">
@@ -3490,19 +3494,19 @@
       </c>
       <c r="C35" s="19" t="n"/>
       <c r="D35" s="47" t="n"/>
-      <c r="E35" s="93" t="n">
+      <c r="E35" s="94" t="n">
         <v>81058</v>
       </c>
-      <c r="F35" s="93" t="n">
+      <c r="F35" s="94" t="n">
         <v>97768</v>
       </c>
-      <c r="G35" s="93" t="n">
+      <c r="G35" s="94" t="n">
         <v>124249</v>
       </c>
-      <c r="H35" s="93" t="n">
+      <c r="H35" s="94" t="n">
         <v>129214</v>
       </c>
-      <c r="I35" s="93" t="n">
+      <c r="I35" s="94" t="n">
         <v>150649</v>
       </c>
       <c r="J35" s="55">
@@ -3631,19 +3635,19 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="E41" s="93" t="n">
+      <c r="E41" s="94" t="n">
         <v>195354</v>
       </c>
-      <c r="F41" s="93" t="n">
+      <c r="F41" s="94" t="n">
         <v>133202</v>
       </c>
-      <c r="G41" s="93" t="n">
+      <c r="G41" s="94" t="n">
         <v>136778</v>
       </c>
-      <c r="H41" s="93" t="n">
+      <c r="H41" s="94" t="n">
         <v>150667</v>
       </c>
-      <c r="I41" s="93" t="n">
+      <c r="I41" s="94" t="n">
         <v>134136</v>
       </c>
       <c r="J41" s="19">
@@ -3673,19 +3677,19 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="E42" s="93" t="n">
+      <c r="E42" s="94" t="n">
         <v>312107</v>
       </c>
-      <c r="F42" s="93" t="n">
+      <c r="F42" s="94" t="n">
         <v>322410</v>
       </c>
-      <c r="G42" s="93" t="n">
+      <c r="G42" s="94" t="n">
         <v>387947</v>
       </c>
-      <c r="H42" s="93" t="n">
+      <c r="H42" s="94" t="n">
         <v>426642</v>
       </c>
-      <c r="I42" s="93" t="n">
+      <c r="I42" s="94" t="n">
         <v>529148</v>
       </c>
       <c r="J42" s="42">
@@ -3715,19 +3719,19 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="E43" s="93" t="n">
+      <c r="E43" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="93" t="n">
+      <c r="F43" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="93" t="n">
+      <c r="G43" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="93" t="n">
+      <c r="H43" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="I43" s="93" t="n">
+      <c r="I43" s="94" t="n">
         <v>0</v>
       </c>
       <c r="J43" s="19">
@@ -3757,19 +3761,19 @@
           <t>Property &amp; Equipment</t>
         </is>
       </c>
-      <c r="E44" s="93" t="n">
+      <c r="E44" s="94" t="n">
         <v>27913</v>
       </c>
-      <c r="F44" s="93" t="n">
+      <c r="F44" s="94" t="n">
         <v>17580</v>
       </c>
-      <c r="G44" s="93" t="n">
+      <c r="G44" s="94" t="n">
         <v>10966</v>
       </c>
-      <c r="H44" s="93" t="n">
+      <c r="H44" s="94" t="n">
         <v>38465</v>
       </c>
-      <c r="I44" s="93" t="n">
+      <c r="I44" s="94" t="n">
         <v>67713</v>
       </c>
       <c r="J44" s="19">
@@ -3875,19 +3879,19 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="E48" s="93" t="n">
+      <c r="E48" s="94" t="n">
         <v>20749</v>
       </c>
-      <c r="F48" s="93" t="n">
+      <c r="F48" s="94" t="n">
         <v>17273</v>
       </c>
-      <c r="G48" s="93" t="n">
+      <c r="G48" s="94" t="n">
         <v>19009</v>
       </c>
-      <c r="H48" s="93" t="n">
+      <c r="H48" s="94" t="n">
         <v>22473</v>
       </c>
-      <c r="I48" s="93" t="n">
+      <c r="I48" s="94" t="n">
         <v>32315</v>
       </c>
       <c r="J48" s="19">
@@ -3917,19 +3921,19 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="E49" s="93" t="n">
+      <c r="E49" s="94" t="n">
         <v>1009018</v>
       </c>
-      <c r="F49" s="93" t="n">
+      <c r="F49" s="94" t="n">
         <v>1823669</v>
       </c>
-      <c r="G49" s="93" t="n">
+      <c r="G49" s="94" t="n">
         <v>1811658</v>
       </c>
-      <c r="H49" s="93" t="n">
+      <c r="H49" s="94" t="n">
         <v>2209021</v>
       </c>
-      <c r="I49" s="93" t="n">
+      <c r="I49" s="94" t="n">
         <v>3055691</v>
       </c>
       <c r="J49" s="19">
@@ -4020,19 +4024,19 @@
           <t>Equity Capital</t>
         </is>
       </c>
-      <c r="E52" s="93" t="n">
+      <c r="E52" s="94" t="n">
         <v>-494393</v>
       </c>
-      <c r="F52" s="93" t="n">
+      <c r="F52" s="94" t="n">
         <v>-1367750</v>
       </c>
-      <c r="G52" s="93" t="n">
+      <c r="G52" s="94" t="n">
         <v>-1294976</v>
       </c>
-      <c r="H52" s="93" t="n">
+      <c r="H52" s="94" t="n">
         <v>-1615720</v>
       </c>
-      <c r="I52" s="93" t="n">
+      <c r="I52" s="94" t="n">
         <v>-2357009</v>
       </c>
       <c r="J52" s="19">
@@ -4062,19 +4066,19 @@
           <t>Retained Earnings</t>
         </is>
       </c>
-      <c r="E53" s="93" t="n">
+      <c r="E53" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="93" t="n">
+      <c r="F53" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="G53" s="93" t="n">
+      <c r="G53" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="93" t="n">
+      <c r="H53" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="I53" s="93" t="n">
+      <c r="I53" s="94" t="n">
         <v>0</v>
       </c>
       <c r="J53" s="19">
@@ -4410,19 +4414,19 @@
           <t>Less: Changes in Working Capital</t>
         </is>
       </c>
-      <c r="E64" s="93" t="n">
+      <c r="E64" s="94" t="n">
         <v>-19789</v>
       </c>
-      <c r="F64" s="93" t="n">
+      <c r="F64" s="94" t="n">
         <v>13779</v>
       </c>
-      <c r="G64" s="93" t="n">
+      <c r="G64" s="94" t="n">
         <v>63801</v>
       </c>
-      <c r="H64" s="93" t="n">
+      <c r="H64" s="94" t="n">
         <v>35231</v>
       </c>
-      <c r="I64" s="93" t="n">
+      <c r="I64" s="94" t="n">
         <v>92664</v>
       </c>
       <c r="J64" s="19">
@@ -4533,19 +4537,19 @@
           <t>Investments in Property &amp; Equipment</t>
         </is>
       </c>
-      <c r="E68" s="93" t="n">
+      <c r="E68" s="94" t="n">
         <v>7569</v>
       </c>
-      <c r="F68" s="93" t="n">
+      <c r="F68" s="94" t="n">
         <v>6029</v>
       </c>
-      <c r="G68" s="93" t="n">
+      <c r="G68" s="94" t="n">
         <v>4237</v>
       </c>
-      <c r="H68" s="93" t="n">
+      <c r="H68" s="94" t="n">
         <v>25551</v>
       </c>
-      <c r="I68" s="93" t="n">
+      <c r="I68" s="94" t="n">
         <v>39407</v>
       </c>
       <c r="J68" s="19">
@@ -4656,19 +4660,19 @@
           <t>Issuance (repayment) of debt</t>
         </is>
       </c>
-      <c r="E72" s="93" t="n">
+      <c r="E72" s="94" t="n">
         <v>269583</v>
       </c>
-      <c r="F72" s="93" t="n">
+      <c r="F72" s="94" t="n">
         <v>814651</v>
       </c>
-      <c r="G72" s="93" t="n">
+      <c r="G72" s="94" t="n">
         <v>-12011</v>
       </c>
-      <c r="H72" s="93" t="n">
+      <c r="H72" s="94" t="n">
         <v>397363</v>
       </c>
-      <c r="I72" s="93" t="n">
+      <c r="I72" s="94" t="n">
         <v>846670</v>
       </c>
       <c r="J72" s="19">
@@ -4698,19 +4702,19 @@
           <t>Issuance (repayment) of equity</t>
         </is>
       </c>
-      <c r="E73" s="93" t="n">
+      <c r="E73" s="94" t="n">
         <v>-661519</v>
       </c>
-      <c r="F73" s="93" t="n">
+      <c r="F73" s="94" t="n">
         <v>-1251001</v>
       </c>
-      <c r="G73" s="93" t="n">
+      <c r="G73" s="94" t="n">
         <v>-360388</v>
       </c>
-      <c r="H73" s="93" t="n">
+      <c r="H73" s="94" t="n">
         <v>-849330</v>
       </c>
-      <c r="I73" s="93" t="n">
+      <c r="I73" s="94" t="n">
         <v>-1398028</v>
       </c>
       <c r="J73" s="19">
@@ -4851,8 +4855,9 @@
           <t>Opening Cash Balance</t>
         </is>
       </c>
-      <c r="E77" s="93" t="n">
-        <v>157394</v>
+      <c r="E77" s="19">
+        <f>D78</f>
+        <v/>
       </c>
       <c r="F77" s="33">
         <f>E78</f>
@@ -4898,7 +4903,9 @@
         </is>
       </c>
       <c r="C78" s="5" t="n"/>
-      <c r="D78" s="28" t="n"/>
+      <c r="D78" s="96" t="n">
+        <v>157394</v>
+      </c>
       <c r="E78" s="17">
         <f>SUM(E76:E77)</f>
         <v/>
@@ -5048,19 +5055,19 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="E85" s="93" t="n">
+      <c r="E85" s="94" t="n">
         <v>312107</v>
       </c>
-      <c r="F85" s="93" t="n">
+      <c r="F85" s="94" t="n">
         <v>322410</v>
       </c>
-      <c r="G85" s="93" t="n">
+      <c r="G85" s="94" t="n">
         <v>387947</v>
       </c>
-      <c r="H85" s="93" t="n">
+      <c r="H85" s="94" t="n">
         <v>426642</v>
       </c>
-      <c r="I85" s="93" t="n">
+      <c r="I85" s="94" t="n">
         <v>529148</v>
       </c>
       <c r="J85" s="19">
@@ -5090,19 +5097,19 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="E86" s="93" t="n">
+      <c r="E86" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="F86" s="93" t="n">
+      <c r="F86" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="G86" s="93" t="n">
+      <c r="G86" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="H86" s="93" t="n">
+      <c r="H86" s="94" t="n">
         <v>0</v>
       </c>
-      <c r="I86" s="93" t="n">
+      <c r="I86" s="94" t="n">
         <v>0</v>
       </c>
       <c r="J86" s="19">
@@ -5132,19 +5139,19 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="E87" s="93" t="n">
+      <c r="E87" s="94" t="n">
         <v>20749</v>
       </c>
-      <c r="F87" s="93" t="n">
+      <c r="F87" s="94" t="n">
         <v>17273</v>
       </c>
-      <c r="G87" s="93" t="n">
+      <c r="G87" s="94" t="n">
         <v>19009</v>
       </c>
-      <c r="H87" s="93" t="n">
+      <c r="H87" s="94" t="n">
         <v>22473</v>
       </c>
-      <c r="I87" s="93" t="n">
+      <c r="I87" s="94" t="n">
         <v>32315</v>
       </c>
       <c r="J87" s="19">
@@ -5289,19 +5296,19 @@
           <t>PPE Opening</t>
         </is>
       </c>
-      <c r="E92" s="93" t="n">
+      <c r="E92" s="94" t="n">
         <v>46419</v>
       </c>
-      <c r="F92" s="93" t="n">
+      <c r="F92" s="94" t="n">
         <v>27913</v>
       </c>
-      <c r="G92" s="93" t="n">
+      <c r="G92" s="94" t="n">
         <v>17580</v>
       </c>
-      <c r="H92" s="93" t="n">
+      <c r="H92" s="94" t="n">
         <v>10966</v>
       </c>
-      <c r="I92" s="93" t="n">
+      <c r="I92" s="94" t="n">
         <v>38465</v>
       </c>
       <c r="J92" s="19">
@@ -5331,19 +5338,19 @@
           <t>Plus Capex</t>
         </is>
       </c>
-      <c r="E93" s="93" t="n">
+      <c r="E93" s="94" t="n">
         <v>7086</v>
       </c>
-      <c r="F93" s="93" t="n">
+      <c r="F93" s="94" t="n">
         <v>10132</v>
       </c>
-      <c r="G93" s="93" t="n">
+      <c r="G93" s="94" t="n">
         <v>8024</v>
       </c>
-      <c r="H93" s="93" t="n">
+      <c r="H93" s="94" t="n">
         <v>41326</v>
       </c>
-      <c r="I93" s="93" t="n">
+      <c r="I93" s="94" t="n">
         <v>44200</v>
       </c>
       <c r="J93" s="19">
@@ -5373,19 +5380,19 @@
           <t>Less Depreciation</t>
         </is>
       </c>
-      <c r="E94" s="93" t="n">
+      <c r="E94" s="94" t="n">
         <v>25592</v>
       </c>
-      <c r="F94" s="93" t="n">
+      <c r="F94" s="94" t="n">
         <v>20465</v>
       </c>
-      <c r="G94" s="93" t="n">
+      <c r="G94" s="94" t="n">
         <v>14638</v>
       </c>
-      <c r="H94" s="93" t="n">
+      <c r="H94" s="94" t="n">
         <v>13827</v>
       </c>
-      <c r="I94" s="93" t="n">
+      <c r="I94" s="94" t="n">
         <v>14952</v>
       </c>
       <c r="J94" s="55">
@@ -5488,19 +5495,19 @@
           <t>Debt Opening</t>
         </is>
       </c>
-      <c r="E98" s="93" t="n">
+      <c r="E98" s="94" t="n">
         <v>739435</v>
       </c>
-      <c r="F98" s="93" t="n">
+      <c r="F98" s="94" t="n">
         <v>1009018</v>
       </c>
-      <c r="G98" s="93" t="n">
+      <c r="G98" s="94" t="n">
         <v>1823669</v>
       </c>
-      <c r="H98" s="93" t="n">
+      <c r="H98" s="94" t="n">
         <v>1811658</v>
       </c>
-      <c r="I98" s="93" t="n">
+      <c r="I98" s="94" t="n">
         <v>2209021</v>
       </c>
       <c r="J98" s="19">
@@ -5530,19 +5537,19 @@
           <t>Issuance (repayment)</t>
         </is>
       </c>
-      <c r="E99" s="93" t="n">
+      <c r="E99" s="94" t="n">
         <v>269583</v>
       </c>
-      <c r="F99" s="93" t="n">
+      <c r="F99" s="94" t="n">
         <v>814651</v>
       </c>
-      <c r="G99" s="93" t="n">
+      <c r="G99" s="94" t="n">
         <v>-12011</v>
       </c>
-      <c r="H99" s="93" t="n">
+      <c r="H99" s="94" t="n">
         <v>397363</v>
       </c>
-      <c r="I99" s="93" t="n">
+      <c r="I99" s="94" t="n">
         <v>846670</v>
       </c>
       <c r="J99" s="52">
@@ -5621,19 +5628,19 @@
           <t>Interest Expense</t>
         </is>
       </c>
-      <c r="E101" s="93" t="n">
+      <c r="E101" s="94" t="n">
         <v>40092</v>
       </c>
-      <c r="F101" s="93" t="n">
+      <c r="F101" s="94" t="n">
         <v>68967</v>
       </c>
-      <c r="G101" s="93" t="n">
+      <c r="G101" s="94" t="n">
         <v>95546</v>
       </c>
-      <c r="H101" s="93" t="n">
+      <c r="H101" s="94" t="n">
         <v>105638</v>
       </c>
-      <c r="I101" s="93" t="n">
+      <c r="I101" s="94" t="n">
         <v>133647</v>
       </c>
       <c r="J101" s="19">
@@ -5884,26 +5891,27 @@
     </row>
     <row r="128" hidden="1" outlineLevel="1"/>
     <row r="129" collapsed="1"/>
+    <row r="130"/>
     <row r="131">
-      <c r="B131" s="95" t="inlineStr">
-        <is>
-          <t>FICO mapping: Revenue/COGS/Interest/Tax from 10-K; SG&amp;A→Salaries; R&amp;D residual→Rent so OpInc identity holds.</t>
+      <c r="B131" s="97" t="inlineStr">
+        <is>
+          <t>FICO SEC mapping: Revenue/COGS/SG&amp;A/R&amp;D/Interest/Tax/Cash/AR/PPE/AP/Debt/D&amp;A/Capex from EDGAR 10-K.</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="B132" s="95" t="inlineStr">
-        <is>
-          <t>Template BS is simplified (Cash/AR/Inv/PPE vs AP/Debt). Equity is a plug. Yellow/blue = inputs.</t>
+      <c r="B132" s="97" t="inlineStr">
+        <is>
+          <t>Yellow/blue = inputs. All subtotals/forecast mechanics remain native CFI formulas.</t>
         </is>
       </c>
       <c r="C132" s="69" t="n"/>
       <c r="D132" s="69" t="n"/>
     </row>
     <row r="133">
-      <c r="B133" s="95" t="inlineStr">
-        <is>
-          <t>Sources: SEC EDGAR FY2025 10-K / companyfacts; forecast drivers are base-case assumptions.</t>
+      <c r="B133" s="97" t="inlineStr">
+        <is>
+          <t>Pulled via SEC companyfacts CIK 0000814547. Units $ thousands. Educational use only.</t>
         </is>
       </c>
       <c r="C133" s="69" t="n"/>

</xml_diff>